<commit_message>
rev 0.3: front panel with I2C OLED, encoder and OUTPUT button
PCF8574 expander (0x20) with INT on GPIO0, 10-pin IDC connector,
RC debounce, I2C pull-ups 2.2k, re-routed PCB (DRC/parity clean),
updated BOM, slides (front panel page) and README.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013KrwoEq2Y4F9LNKutY5RJ4
</commit_message>
<xml_diff>
--- a/hardware/bom/eload_4ch_bom_priced.xlsx
+++ b/hardware/bom/eload_4ch_bom_priced.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Parametri" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">BOM!$A$4:$O$52</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">BOM!$A$4:$O$56</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,9 +25,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="268">
-  <si>
-    <t xml:space="preserve">BOM con prezzi — Carico attivo 60 V / 20 A / 300 W, 4 canali (controllo WiFi Wemos D1 mini Pro) — rev 0.2</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="290">
+  <si>
+    <t xml:space="preserve">BOM con prezzi — Carico attivo 60 V / 20 A / 300 W, 4 canali (controllo WiFi Wemos D1 mini Pro) — rev 0.3</t>
   </si>
   <si>
     <t xml:space="preserve">Prezzi IVA esclusa, a quantità singola. Celle blu = valori inseriti a mano; cambi e numero di schede nel foglio Parametri.</t>
@@ -123,7 +123,7 @@
     <t xml:space="preserve">stima</t>
   </si>
   <si>
-    <t xml:space="preserve">C3,C4,C7,C10,C13,C16,C20,C22,C23,C25-C27,C29</t>
+    <t xml:space="preserve">C3,C4,C7,C10,C13,C16,C20,C22,C28-C30,C32-C34,C36</t>
   </si>
   <si>
     <t xml:space="preserve">100n</t>
@@ -159,7 +159,7 @@
     <t xml:space="preserve">Compensazione loop (rev 0.2)</t>
   </si>
   <si>
-    <t xml:space="preserve">C17,C18,C33,C34</t>
+    <t xml:space="preserve">C17,C18,C40,C41</t>
   </si>
   <si>
     <t xml:space="preserve">100n 50V</t>
@@ -168,7 +168,7 @@
     <t xml:space="preserve">1206B104K500CT (Walsin)</t>
   </si>
   <si>
-    <t xml:space="preserve">C19,C21,C28,C31,C32</t>
+    <t xml:space="preserve">C19,C21,C27,C35,C38,C39</t>
   </si>
   <si>
     <t xml:space="preserve">10u 25V</t>
@@ -183,7 +183,7 @@
     <t xml:space="preserve">Prezzo a 10 pz, parte da 50 V</t>
   </si>
   <si>
-    <t xml:space="preserve">C24,C30</t>
+    <t xml:space="preserve">C31,C37</t>
   </si>
   <si>
     <t xml:space="preserve">1u</t>
@@ -192,7 +192,16 @@
     <t xml:space="preserve">generico X7R 50V</t>
   </si>
   <si>
-    <t xml:space="preserve">C35,C36</t>
+    <t xml:space="preserve">C23-C26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Antirimbalzo pannello (rev 0.3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C42,C43</t>
   </si>
   <si>
     <t xml:space="preserve">22u 10V</t>
@@ -369,7 +378,19 @@
     <t xml:space="preserve">Zoccolo per il Wemos</t>
   </si>
   <si>
-    <t xml:space="preserve">J6,J7</t>
+    <t xml:space="preserve">J6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Header IDC 2x5 2,54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDC-Header 2x05 verticale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pannello frontale (rev 0.3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J7,J8</t>
   </si>
   <si>
     <t xml:space="preserve">Molex KK 4 vie</t>
@@ -378,7 +399,7 @@
     <t xml:space="preserve">22-27-2041</t>
   </si>
   <si>
-    <t xml:space="preserve">J8</t>
+    <t xml:space="preserve">J9</t>
   </si>
   <si>
     <t xml:space="preserve">Jack DC</t>
@@ -465,13 +486,13 @@
     <t xml:space="preserve">Resistori</t>
   </si>
   <si>
-    <t xml:space="preserve">R1,R15,R21,R27,R33,R44</t>
+    <t xml:space="preserve">R1,R15,R21,R27,R33,R49</t>
   </si>
   <si>
     <t xml:space="preserve">100R 1%</t>
   </si>
   <si>
-    <t xml:space="preserve">R2,R5,R8,R16,R22,R28,R34,R39,R41,R43,R46</t>
+    <t xml:space="preserve">R2,R5,R8,R16,R22,R28,R34,R39-R42,R44,R46,R48,R51</t>
   </si>
   <si>
     <t xml:space="preserve">10k 1%</t>
@@ -483,7 +504,7 @@
     <t xml:space="preserve">10R 1%</t>
   </si>
   <si>
-    <t xml:space="preserve">R4,R14,R20,R26,R32,R36,R40</t>
+    <t xml:space="preserve">R4,R14,R20,R26,R32,R36,R45</t>
   </si>
   <si>
     <t xml:space="preserve">1k 1%</t>
@@ -504,7 +525,7 @@
     <t xml:space="preserve">generico (≥200 V)</t>
   </si>
   <si>
-    <t xml:space="preserve">R10,R42,R45,R50</t>
+    <t xml:space="preserve">R10,R47,R50,R55</t>
   </si>
   <si>
     <t xml:space="preserve">100k 1%</t>
@@ -561,10 +582,19 @@
     <t xml:space="preserve">R37,R38</t>
   </si>
   <si>
-    <t xml:space="preserve">4k7 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R47,R48</t>
+    <t xml:space="preserve">2k2 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">470R 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LED OUTPUT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R52,R53</t>
   </si>
   <si>
     <t xml:space="preserve">10k 0,1%</t>
@@ -573,7 +603,7 @@
     <t xml:space="preserve">thin film 0,1%</t>
   </si>
   <si>
-    <t xml:space="preserve">R49</t>
+    <t xml:space="preserve">R54</t>
   </si>
   <si>
     <t xml:space="preserve">1k5 1%</t>
@@ -636,6 +666,21 @@
     <t xml:space="preserve">U9</t>
   </si>
   <si>
+    <t xml:space="preserve">Espansore I/O I2C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOIC-16W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PCF8574T/3 (NXP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">@0x20, pannello frontale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U10</t>
+  </si>
+  <si>
     <t xml:space="preserve">DAC 4ch 16 bit</t>
   </si>
   <si>
@@ -651,7 +696,7 @@
     <t xml:space="preserve">LCSC: IAPWR 11,80 USD ma NRND</t>
   </si>
   <si>
-    <t xml:space="preserve">U10</t>
+    <t xml:space="preserve">U11</t>
   </si>
   <si>
     <t xml:space="preserve">LDO 5V 100mA (analogico)</t>
@@ -660,7 +705,7 @@
     <t xml:space="preserve">L78L05ACD13TR</t>
   </si>
   <si>
-    <t xml:space="preserve">U11</t>
+    <t xml:space="preserve">U12</t>
   </si>
   <si>
     <t xml:space="preserve">Buck 5V 2A</t>
@@ -766,6 +811,27 @@
   </si>
   <si>
     <t xml:space="preserve">Alimentatore 12 V ≥ 2 A con jack 5,5/2,1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pannello frontale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OLED 2,42" 128x64 I2C (SSD1309) o 1,3" SH1106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indirizzo 0x3C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Encoder EC11 con pulsante + manopola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pulsante OUTPUT con LED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flat 10 poli + 2 connettori IDC 2x5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max ~20 cm</t>
   </si>
   <si>
     <t xml:space="preserve">Antenna 2,4 GHz con cavetto U.FL (opzionale, se il case è metallico)</t>
@@ -1415,7 +1481,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O72"/>
+  <dimension ref="A1:O76"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -1595,7 +1661,7 @@
         <v>32</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>33</v>
@@ -1621,11 +1687,11 @@
       </c>
       <c r="K7" s="4" t="n">
         <f aca="false">C7*Parametri!$B$7</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="L7" s="9" t="n">
         <f aca="false">IF(J7="","",J7*K7)</f>
-        <v>0.1677</v>
+        <v>0.1935</v>
       </c>
       <c r="M7" s="11" t="s">
         <v>31</v>
@@ -1789,7 +1855,7 @@
         <v>47</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>48</v>
@@ -1815,11 +1881,11 @@
       </c>
       <c r="K11" s="4" t="n">
         <f aca="false">C11*Parametri!$B$7</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L11" s="9" t="n">
         <f aca="false">IF(J11="","",J11*K11)</f>
-        <v>0.28681</v>
+        <v>0.344172</v>
       </c>
       <c r="M11" s="4" t="s">
         <v>24</v>
@@ -1885,7 +1951,7 @@
         <v>55</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D13" s="4" t="s">
         <v>56</v>
@@ -1894,118 +1960,116 @@
         <v>20</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="G13" s="4" t="s">
         <v>30</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="I13" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J13" s="8" t="n">
         <f aca="false">IF(H13="","",H13*IF(I13="USD",Parametri!$B$3,IF(I13="GBP",Parametri!$B$4,IF(I13="CNY",Parametri!$B$5,1))))</f>
-        <v>0.043</v>
+        <v>0.0086</v>
       </c>
       <c r="K13" s="4" t="n">
         <f aca="false">C13*Parametri!$B$7</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L13" s="9" t="n">
         <f aca="false">IF(J13="","",J13*K13)</f>
-        <v>0.086</v>
+        <v>0.0344</v>
       </c>
       <c r="M13" s="11" t="s">
         <v>31</v>
       </c>
       <c r="N13" s="4"/>
       <c r="O13" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="E14" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="5" t="s">
         <v>60</v>
-      </c>
-      <c r="C14" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>63</v>
       </c>
       <c r="G14" s="4" t="s">
         <v>30</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>3.5052</v>
+        <v>0.05</v>
       </c>
       <c r="I14" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J14" s="8" t="n">
         <f aca="false">IF(H14="","",H14*IF(I14="USD",Parametri!$B$3,IF(I14="GBP",Parametri!$B$4,IF(I14="CNY",Parametri!$B$5,1))))</f>
-        <v>3.014472</v>
+        <v>0.043</v>
       </c>
       <c r="K14" s="4" t="n">
         <f aca="false">C14*Parametri!$B$7</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L14" s="9" t="n">
         <f aca="false">IF(J14="","",J14*K14)</f>
-        <v>3.014472</v>
-      </c>
-      <c r="M14" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="N14" s="10" t="s">
-        <v>64</v>
-      </c>
+        <v>0.086</v>
+      </c>
+      <c r="M14" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="N14" s="4"/>
       <c r="O14" s="5" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B15" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="F15" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="C15" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>69</v>
       </c>
       <c r="G15" s="4" t="s">
         <v>30</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>0.25</v>
+        <v>3.5052</v>
       </c>
       <c r="I15" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J15" s="8" t="n">
         <f aca="false">IF(H15="","",H15*IF(I15="USD",Parametri!$B$3,IF(I15="GBP",Parametri!$B$4,IF(I15="CNY",Parametri!$B$5,1))))</f>
-        <v>0.215</v>
+        <v>3.014472</v>
       </c>
       <c r="K15" s="4" t="n">
         <f aca="false">C15*Parametri!$B$7</f>
@@ -2013,45 +2077,49 @@
       </c>
       <c r="L15" s="9" t="n">
         <f aca="false">IF(J15="","",J15*K15)</f>
-        <v>0.215</v>
-      </c>
-      <c r="M15" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="N15" s="4"/>
-      <c r="O15" s="5"/>
+        <v>3.014472</v>
+      </c>
+      <c r="M15" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="N15" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="O15" s="5" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B16" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="C16" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="4" t="s">
+      <c r="E16" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="F16" s="5" t="s">
         <v>72</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>73</v>
       </c>
       <c r="G16" s="4" t="s">
         <v>30</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>0.08</v>
+        <v>0.25</v>
       </c>
       <c r="I16" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J16" s="8" t="n">
         <f aca="false">IF(H16="","",H16*IF(I16="USD",Parametri!$B$3,IF(I16="GBP",Parametri!$B$4,IF(I16="CNY",Parametri!$B$5,1))))</f>
-        <v>0.0688</v>
+        <v>0.215</v>
       </c>
       <c r="K16" s="4" t="n">
         <f aca="false">C16*Parametri!$B$7</f>
@@ -2059,7 +2127,7 @@
       </c>
       <c r="L16" s="9" t="n">
         <f aca="false">IF(J16="","",J16*K16)</f>
-        <v>0.0688</v>
+        <v>0.215</v>
       </c>
       <c r="M16" s="11" t="s">
         <v>31</v>
@@ -2069,19 +2137,19 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B17" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="C17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="4" t="s">
+      <c r="E17" s="4" t="s">
         <v>75</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>72</v>
       </c>
       <c r="F17" s="5" t="s">
         <v>76</v>
@@ -2090,14 +2158,14 @@
         <v>30</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>0.03</v>
+        <v>0.08</v>
       </c>
       <c r="I17" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J17" s="8" t="n">
         <f aca="false">IF(H17="","",H17*IF(I17="USD",Parametri!$B$3,IF(I17="GBP",Parametri!$B$4,IF(I17="CNY",Parametri!$B$5,1))))</f>
-        <v>0.0258</v>
+        <v>0.0688</v>
       </c>
       <c r="K17" s="4" t="n">
         <f aca="false">C17*Parametri!$B$7</f>
@@ -2105,7 +2173,7 @@
       </c>
       <c r="L17" s="9" t="n">
         <f aca="false">IF(J17="","",J17*K17)</f>
-        <v>0.0258</v>
+        <v>0.0688</v>
       </c>
       <c r="M17" s="11" t="s">
         <v>31</v>
@@ -2115,7 +2183,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>77</v>
@@ -2127,7 +2195,7 @@
         <v>78</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="F18" s="5" t="s">
         <v>79</v>
@@ -2161,35 +2229,35 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="C19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="4" t="s">
+      <c r="E19" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F19" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="E19" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>84</v>
-      </c>
       <c r="G19" s="4" t="s">
-        <v>85</v>
+        <v>30</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>0.235</v>
+        <v>0.03</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>86</v>
+        <v>23</v>
       </c>
       <c r="J19" s="8" t="n">
         <f aca="false">IF(H19="","",H19*IF(I19="USD",Parametri!$B$3,IF(I19="GBP",Parametri!$B$4,IF(I19="CNY",Parametri!$B$5,1))))</f>
-        <v>0.27025</v>
+        <v>0.0258</v>
       </c>
       <c r="K19" s="4" t="n">
         <f aca="false">C19*Parametri!$B$7</f>
@@ -2197,253 +2265,251 @@
       </c>
       <c r="L19" s="9" t="n">
         <f aca="false">IF(J19="","",J19*K19)</f>
-        <v>0.27025</v>
-      </c>
-      <c r="M19" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="N19" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="O19" s="5" t="s">
-        <v>88</v>
-      </c>
+        <v>0.0258</v>
+      </c>
+      <c r="M19" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="N19" s="4"/>
+      <c r="O19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B20" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="H20" s="7" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="I20" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="C20" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="G20" s="4"/>
-      <c r="H20" s="7"/>
-      <c r="I20" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="J20" s="8" t="str">
+      <c r="J20" s="8" t="n">
         <f aca="false">IF(H20="","",H20*IF(I20="USD",Parametri!$B$3,IF(I20="GBP",Parametri!$B$4,IF(I20="CNY",Parametri!$B$5,1))))</f>
-        <v/>
+        <v>0.27025</v>
       </c>
       <c r="K20" s="4" t="n">
         <f aca="false">C20*Parametri!$B$7</f>
         <v>1</v>
       </c>
-      <c r="L20" s="9" t="str">
+      <c r="L20" s="9" t="n">
         <f aca="false">IF(J20="","",J20*K20)</f>
+        <v>0.27025</v>
+      </c>
+      <c r="M20" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="N20" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="O20" s="5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="G21" s="4"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="J21" s="8" t="str">
+        <f aca="false">IF(H21="","",H21*IF(I21="USD",Parametri!$B$3,IF(I21="GBP",Parametri!$B$4,IF(I21="CNY",Parametri!$B$5,1))))</f>
         <v/>
-      </c>
-      <c r="M20" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="N20" s="4"/>
-      <c r="O20" s="5" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="C21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="G21" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="H21" s="7" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I21" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="J21" s="8" t="n">
-        <f aca="false">IF(H21="","",H21*IF(I21="USD",Parametri!$B$3,IF(I21="GBP",Parametri!$B$4,IF(I21="CNY",Parametri!$B$5,1))))</f>
-        <v>0.129</v>
       </c>
       <c r="K21" s="4" t="n">
         <f aca="false">C21*Parametri!$B$7</f>
         <v>1</v>
       </c>
-      <c r="L21" s="9" t="n">
+      <c r="L21" s="9" t="str">
         <f aca="false">IF(J21="","",J21*K21)</f>
-        <v>0.129</v>
-      </c>
-      <c r="M21" s="11" t="s">
-        <v>31</v>
+        <v/>
+      </c>
+      <c r="M21" s="12" t="s">
+        <v>97</v>
       </c>
       <c r="N21" s="4"/>
       <c r="O21" s="5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B22" s="5" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+      <c r="C22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="E22" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F22" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="C22" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>104</v>
-      </c>
       <c r="G22" s="4" t="s">
-        <v>105</v>
+        <v>30</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>0.6</v>
+        <v>0.15</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>93</v>
+        <v>23</v>
       </c>
       <c r="J22" s="8" t="n">
         <f aca="false">IF(H22="","",H22*IF(I22="USD",Parametri!$B$3,IF(I22="GBP",Parametri!$B$4,IF(I22="CNY",Parametri!$B$5,1))))</f>
-        <v>0.6</v>
+        <v>0.129</v>
       </c>
       <c r="K22" s="4" t="n">
         <f aca="false">C22*Parametri!$B$7</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L22" s="9" t="n">
         <f aca="false">IF(J22="","",J22*K22)</f>
-        <v>1.2</v>
+        <v>0.129</v>
       </c>
       <c r="M22" s="11" t="s">
         <v>31</v>
       </c>
       <c r="N22" s="4"/>
       <c r="O22" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E23" s="4" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="B23" s="5" t="s">
+      <c r="F23" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="C23" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="4" t="s">
+      <c r="G23" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="E23" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="F23" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="G23" s="4"/>
       <c r="H23" s="7" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="J23" s="8" t="n">
         <f aca="false">IF(H23="","",H23*IF(I23="USD",Parametri!$B$3,IF(I23="GBP",Parametri!$B$4,IF(I23="CNY",Parametri!$B$5,1))))</f>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="K23" s="4" t="n">
         <f aca="false">C23*Parametri!$B$7</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L23" s="9" t="n">
         <f aca="false">IF(J23="","",J23*K23)</f>
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
       <c r="M23" s="11" t="s">
         <v>31</v>
       </c>
       <c r="N23" s="4"/>
-      <c r="O23" s="5"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O23" s="5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B24" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="C24" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D24" s="4" t="s">
+      <c r="E24" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="E24" s="4" t="s">
-        <v>109</v>
-      </c>
       <c r="F24" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="G24" s="4" t="s">
-        <v>30</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="G24" s="4"/>
       <c r="H24" s="7" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J24" s="8" t="n">
         <f aca="false">IF(H24="","",H24*IF(I24="USD",Parametri!$B$3,IF(I24="GBP",Parametri!$B$4,IF(I24="CNY",Parametri!$B$5,1))))</f>
-        <v>0.258</v>
+        <v>0.8</v>
       </c>
       <c r="K24" s="4" t="n">
         <f aca="false">C24*Parametri!$B$7</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L24" s="9" t="n">
         <f aca="false">IF(J24="","",J24*K24)</f>
-        <v>0.516</v>
+        <v>0.8</v>
       </c>
       <c r="M24" s="11" t="s">
         <v>31</v>
       </c>
       <c r="N24" s="4"/>
-      <c r="O24" s="5" t="s">
-        <v>113</v>
-      </c>
+      <c r="O24" s="5"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>114</v>
@@ -2455,21 +2521,23 @@
         <v>115</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="G25" s="4"/>
+        <v>82</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>30</v>
+      </c>
       <c r="H25" s="7" t="n">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="I25" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J25" s="8" t="n">
         <f aca="false">IF(H25="","",H25*IF(I25="USD",Parametri!$B$3,IF(I25="GBP",Parametri!$B$4,IF(I25="CNY",Parametri!$B$5,1))))</f>
-        <v>0.301</v>
+        <v>0.258</v>
       </c>
       <c r="K25" s="4" t="n">
         <f aca="false">C25*Parametri!$B$7</f>
@@ -2477,17 +2545,19 @@
       </c>
       <c r="L25" s="9" t="n">
         <f aca="false">IF(J25="","",J25*K25)</f>
-        <v>0.602</v>
+        <v>0.516</v>
       </c>
       <c r="M25" s="11" t="s">
         <v>31</v>
       </c>
       <c r="N25" s="4"/>
-      <c r="O25" s="5"/>
+      <c r="O25" s="5" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>117</v>
@@ -2499,21 +2569,23 @@
         <v>118</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="F26" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="G26" s="4"/>
+      <c r="G26" s="4" t="s">
+        <v>30</v>
+      </c>
       <c r="H26" s="7" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="I26" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J26" s="8" t="n">
         <f aca="false">IF(H26="","",H26*IF(I26="USD",Parametri!$B$3,IF(I26="GBP",Parametri!$B$4,IF(I26="CNY",Parametri!$B$5,1))))</f>
-        <v>0.516</v>
+        <v>0.258</v>
       </c>
       <c r="K26" s="4" t="n">
         <f aca="false">C26*Parametri!$B$7</f>
@@ -2521,93 +2593,89 @@
       </c>
       <c r="L26" s="9" t="n">
         <f aca="false">IF(J26="","",J26*K26)</f>
-        <v>0.516</v>
+        <v>0.258</v>
       </c>
       <c r="M26" s="11" t="s">
         <v>31</v>
       </c>
       <c r="N26" s="4"/>
-      <c r="O26" s="5"/>
-    </row>
-    <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O26" s="5" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>120</v>
+        <v>103</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>121</v>
       </c>
       <c r="C27" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>122</v>
       </c>
       <c r="E27" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="F27" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="F27" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="G27" s="4" t="s">
-        <v>125</v>
-      </c>
+      <c r="G27" s="4"/>
       <c r="H27" s="7" t="n">
-        <v>7.44</v>
+        <v>0.35</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>93</v>
+        <v>23</v>
       </c>
       <c r="J27" s="8" t="n">
         <f aca="false">IF(H27="","",H27*IF(I27="USD",Parametri!$B$3,IF(I27="GBP",Parametri!$B$4,IF(I27="CNY",Parametri!$B$5,1))))</f>
-        <v>7.44</v>
+        <v>0.301</v>
       </c>
       <c r="K27" s="4" t="n">
         <f aca="false">C27*Parametri!$B$7</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L27" s="9" t="n">
         <f aca="false">IF(J27="","",J27*K27)</f>
-        <v>7.44</v>
-      </c>
-      <c r="M27" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="N27" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="O27" s="5" t="s">
-        <v>127</v>
-      </c>
+        <v>0.602</v>
+      </c>
+      <c r="M27" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="N27" s="4"/>
+      <c r="O27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>128</v>
+        <v>103</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="C28" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>131</v>
+        <v>112</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="G28" s="4"/>
       <c r="H28" s="7" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
       <c r="I28" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J28" s="8" t="n">
         <f aca="false">IF(H28="","",H28*IF(I28="USD",Parametri!$B$3,IF(I28="GBP",Parametri!$B$4,IF(I28="CNY",Parametri!$B$5,1))))</f>
-        <v>0.258</v>
+        <v>0.516</v>
       </c>
       <c r="K28" s="4" t="n">
         <f aca="false">C28*Parametri!$B$7</f>
@@ -2615,7 +2683,7 @@
       </c>
       <c r="L28" s="9" t="n">
         <f aca="false">IF(J28="","",J28*K28)</f>
-        <v>0.258</v>
+        <v>0.516</v>
       </c>
       <c r="M28" s="11" t="s">
         <v>31</v>
@@ -2625,91 +2693,91 @@
     </row>
     <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="C29" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>17.59</v>
+        <v>7.44</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J29" s="8" t="n">
         <f aca="false">IF(H29="","",H29*IF(I29="USD",Parametri!$B$3,IF(I29="GBP",Parametri!$B$4,IF(I29="CNY",Parametri!$B$5,1))))</f>
-        <v>15.1274</v>
+        <v>7.44</v>
       </c>
       <c r="K29" s="4" t="n">
         <f aca="false">C29*Parametri!$B$7</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L29" s="9" t="n">
         <f aca="false">IF(J29="","",J29*K29)</f>
-        <v>60.5096</v>
+        <v>7.44</v>
       </c>
       <c r="M29" s="4" t="s">
         <v>24</v>
       </c>
       <c r="N29" s="10" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="O29" s="5" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C30" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="G30" s="4"/>
       <c r="H30" s="7" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="I30" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J30" s="8" t="n">
         <f aca="false">IF(H30="","",H30*IF(I30="USD",Parametri!$B$3,IF(I30="GBP",Parametri!$B$4,IF(I30="CNY",Parametri!$B$5,1))))</f>
-        <v>0.344</v>
+        <v>0.258</v>
       </c>
       <c r="K30" s="4" t="n">
         <f aca="false">C30*Parametri!$B$7</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L30" s="9" t="n">
         <f aca="false">IF(J30="","",J30*K30)</f>
-        <v>1.032</v>
+        <v>0.258</v>
       </c>
       <c r="M30" s="11" t="s">
         <v>31</v>
@@ -2717,91 +2785,93 @@
       <c r="N30" s="4"/>
       <c r="O30" s="5"/>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="G31" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="B31" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="C31" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="G31" s="4" t="s">
-        <v>30</v>
-      </c>
       <c r="H31" s="7" t="n">
-        <v>0.005</v>
+        <v>17.59</v>
       </c>
       <c r="I31" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J31" s="8" t="n">
         <f aca="false">IF(H31="","",H31*IF(I31="USD",Parametri!$B$3,IF(I31="GBP",Parametri!$B$4,IF(I31="CNY",Parametri!$B$5,1))))</f>
-        <v>0.0043</v>
+        <v>15.1274</v>
       </c>
       <c r="K31" s="4" t="n">
         <f aca="false">C31*Parametri!$B$7</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L31" s="9" t="n">
         <f aca="false">IF(J31="","",J31*K31)</f>
-        <v>0.0258</v>
-      </c>
-      <c r="M31" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="N31" s="4"/>
-      <c r="O31" s="5"/>
-    </row>
-    <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>60.5096</v>
+      </c>
+      <c r="M31" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="N31" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="O31" s="5" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>148</v>
       </c>
       <c r="C32" s="6" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>149</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="G32" s="4" t="s">
-        <v>30</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="G32" s="4"/>
       <c r="H32" s="7" t="n">
-        <v>0.005</v>
+        <v>0.4</v>
       </c>
       <c r="I32" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J32" s="8" t="n">
         <f aca="false">IF(H32="","",H32*IF(I32="USD",Parametri!$B$3,IF(I32="GBP",Parametri!$B$4,IF(I32="CNY",Parametri!$B$5,1))))</f>
-        <v>0.0043</v>
+        <v>0.344</v>
       </c>
       <c r="K32" s="4" t="n">
         <f aca="false">C32*Parametri!$B$7</f>
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="L32" s="9" t="n">
         <f aca="false">IF(J32="","",J32*K32)</f>
-        <v>0.0473</v>
+        <v>1.032</v>
       </c>
       <c r="M32" s="11" t="s">
         <v>31</v>
@@ -2811,22 +2881,22 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C33" s="6" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>20</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="G33" s="4" t="s">
         <v>30</v>
@@ -2843,11 +2913,11 @@
       </c>
       <c r="K33" s="4" t="n">
         <f aca="false">C33*Parametri!$B$7</f>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L33" s="9" t="n">
         <f aca="false">IF(J33="","",J33*K33)</f>
-        <v>0.0043</v>
+        <v>0.0258</v>
       </c>
       <c r="M33" s="11" t="s">
         <v>31</v>
@@ -2855,24 +2925,24 @@
       <c r="N33" s="4"/>
       <c r="O33" s="5"/>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C34" s="6" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="E34" s="4" t="s">
         <v>20</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="G34" s="4" t="s">
         <v>30</v>
@@ -2889,11 +2959,11 @@
       </c>
       <c r="K34" s="4" t="n">
         <f aca="false">C34*Parametri!$B$7</f>
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="L34" s="9" t="n">
         <f aca="false">IF(J34="","",J34*K34)</f>
-        <v>0.0301</v>
+        <v>0.0645</v>
       </c>
       <c r="M34" s="11" t="s">
         <v>31</v>
@@ -2903,22 +2973,22 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="C35" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>20</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="G35" s="4" t="s">
         <v>30</v>
@@ -2935,11 +3005,11 @@
       </c>
       <c r="K35" s="4" t="n">
         <f aca="false">C35*Parametri!$B$7</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L35" s="9" t="n">
         <f aca="false">IF(J35="","",J35*K35)</f>
-        <v>0.0086</v>
+        <v>0.0043</v>
       </c>
       <c r="M35" s="11" t="s">
         <v>31</v>
@@ -2949,22 +3019,22 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C36" s="6" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E36" s="4" t="s">
         <v>20</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>158</v>
+        <v>82</v>
       </c>
       <c r="G36" s="4" t="s">
         <v>30</v>
@@ -2981,11 +3051,11 @@
       </c>
       <c r="K36" s="4" t="n">
         <f aca="false">C36*Parametri!$B$7</f>
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L36" s="9" t="n">
         <f aca="false">IF(J36="","",J36*K36)</f>
-        <v>0.0043</v>
+        <v>0.0301</v>
       </c>
       <c r="M36" s="11" t="s">
         <v>31</v>
@@ -2995,22 +3065,22 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C37" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E37" s="4" t="s">
         <v>20</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="G37" s="4" t="s">
         <v>30</v>
@@ -3027,11 +3097,11 @@
       </c>
       <c r="K37" s="4" t="n">
         <f aca="false">C37*Parametri!$B$7</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L37" s="9" t="n">
         <f aca="false">IF(J37="","",J37*K37)</f>
-        <v>0.0172</v>
+        <v>0.0086</v>
       </c>
       <c r="M37" s="11" t="s">
         <v>31</v>
@@ -3041,22 +3111,22 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C38" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E38" s="4" t="s">
         <v>20</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>79</v>
+        <v>165</v>
       </c>
       <c r="G38" s="4" t="s">
         <v>30</v>
@@ -3087,35 +3157,35 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C39" s="6" t="n">
         <v>4</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="E39" s="4" t="s">
         <v>20</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>165</v>
+        <v>82</v>
       </c>
       <c r="G39" s="4" t="s">
         <v>30</v>
       </c>
       <c r="H39" s="7" t="n">
-        <v>0.25</v>
+        <v>0.005</v>
       </c>
       <c r="I39" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J39" s="8" t="n">
         <f aca="false">IF(H39="","",H39*IF(I39="USD",Parametri!$B$3,IF(I39="GBP",Parametri!$B$4,IF(I39="CNY",Parametri!$B$5,1))))</f>
-        <v>0.215</v>
+        <v>0.0043</v>
       </c>
       <c r="K39" s="4" t="n">
         <f aca="false">C39*Parametri!$B$7</f>
@@ -3123,55 +3193,53 @@
       </c>
       <c r="L39" s="9" t="n">
         <f aca="false">IF(J39="","",J39*K39)</f>
-        <v>0.86</v>
+        <v>0.0172</v>
       </c>
       <c r="M39" s="11" t="s">
         <v>31</v>
       </c>
       <c r="N39" s="4"/>
-      <c r="O39" s="5" t="s">
-        <v>166</v>
-      </c>
+      <c r="O39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C40" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E40" s="4" t="s">
         <v>20</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>165</v>
+        <v>82</v>
       </c>
       <c r="G40" s="4" t="s">
         <v>30</v>
       </c>
       <c r="H40" s="7" t="n">
-        <v>0.25</v>
+        <v>0.005</v>
       </c>
       <c r="I40" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J40" s="8" t="n">
         <f aca="false">IF(H40="","",H40*IF(I40="USD",Parametri!$B$3,IF(I40="GBP",Parametri!$B$4,IF(I40="CNY",Parametri!$B$5,1))))</f>
-        <v>0.215</v>
+        <v>0.0043</v>
       </c>
       <c r="K40" s="4" t="n">
         <f aca="false">C40*Parametri!$B$7</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L40" s="9" t="n">
         <f aca="false">IF(J40="","",J40*K40)</f>
-        <v>0.86</v>
+        <v>0.0043</v>
       </c>
       <c r="M40" s="11" t="s">
         <v>31</v>
@@ -3179,37 +3247,37 @@
       <c r="N40" s="4"/>
       <c r="O40" s="5"/>
     </row>
-    <row r="41" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C41" s="6" t="n">
         <v>4</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>171</v>
+        <v>20</v>
       </c>
       <c r="F41" s="5" t="s">
         <v>172</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>173</v>
+        <v>30</v>
       </c>
       <c r="H41" s="7" t="n">
-        <v>23.72</v>
+        <v>0.25</v>
       </c>
       <c r="I41" s="6" t="s">
-        <v>174</v>
+        <v>23</v>
       </c>
       <c r="J41" s="8" t="n">
         <f aca="false">IF(H41="","",H41*IF(I41="USD",Parametri!$B$3,IF(I41="GBP",Parametri!$B$4,IF(I41="CNY",Parametri!$B$5,1))))</f>
-        <v>2.8464</v>
+        <v>0.215</v>
       </c>
       <c r="K41" s="4" t="n">
         <f aca="false">C41*Parametri!$B$7</f>
@@ -3217,57 +3285,55 @@
       </c>
       <c r="L41" s="9" t="n">
         <f aca="false">IF(J41="","",J41*K41)</f>
-        <v>11.3856</v>
-      </c>
-      <c r="M41" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="N41" s="10" t="s">
-        <v>175</v>
-      </c>
+        <v>0.86</v>
+      </c>
+      <c r="M41" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="N41" s="4"/>
       <c r="O41" s="5" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="C42" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="E42" s="4" t="s">
         <v>20</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>79</v>
+        <v>172</v>
       </c>
       <c r="G42" s="4" t="s">
         <v>30</v>
       </c>
       <c r="H42" s="7" t="n">
-        <v>0.005</v>
+        <v>0.25</v>
       </c>
       <c r="I42" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J42" s="8" t="n">
         <f aca="false">IF(H42="","",H42*IF(I42="USD",Parametri!$B$3,IF(I42="GBP",Parametri!$B$4,IF(I42="CNY",Parametri!$B$5,1))))</f>
-        <v>0.0043</v>
+        <v>0.215</v>
       </c>
       <c r="K42" s="4" t="n">
         <f aca="false">C42*Parametri!$B$7</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L42" s="9" t="n">
         <f aca="false">IF(J42="","",J42*K42)</f>
-        <v>0.0086</v>
+        <v>0.86</v>
       </c>
       <c r="M42" s="11" t="s">
         <v>31</v>
@@ -3275,70 +3341,74 @@
       <c r="N42" s="4"/>
       <c r="O42" s="5"/>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B43" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="C43" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="F43" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="C43" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D43" s="4" t="s">
+      <c r="G43" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="E43" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F43" s="5" t="s">
+      <c r="H43" s="7" t="n">
+        <v>23.72</v>
+      </c>
+      <c r="I43" s="6" t="s">
         <v>181</v>
-      </c>
-      <c r="G43" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="H43" s="7" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="I43" s="6" t="s">
-        <v>23</v>
       </c>
       <c r="J43" s="8" t="n">
         <f aca="false">IF(H43="","",H43*IF(I43="USD",Parametri!$B$3,IF(I43="GBP",Parametri!$B$4,IF(I43="CNY",Parametri!$B$5,1))))</f>
-        <v>0.215</v>
+        <v>2.8464</v>
       </c>
       <c r="K43" s="4" t="n">
         <f aca="false">C43*Parametri!$B$7</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L43" s="9" t="n">
         <f aca="false">IF(J43="","",J43*K43)</f>
-        <v>0.43</v>
-      </c>
-      <c r="M43" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="N43" s="4"/>
-      <c r="O43" s="5"/>
+        <v>11.3856</v>
+      </c>
+      <c r="M43" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="N43" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="O43" s="5" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C44" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="E44" s="4" t="s">
         <v>20</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="G44" s="4" t="s">
         <v>30</v>
@@ -3355,11 +3425,11 @@
       </c>
       <c r="K44" s="4" t="n">
         <f aca="false">C44*Parametri!$B$7</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L44" s="9" t="n">
         <f aca="false">IF(J44="","",J44*K44)</f>
-        <v>0.0043</v>
+        <v>0.0086</v>
       </c>
       <c r="M44" s="11" t="s">
         <v>31</v>
@@ -3369,33 +3439,35 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
-        <v>184</v>
+        <v>152</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C45" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>143</v>
+        <v>20</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="G45" s="4"/>
+        <v>82</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>30</v>
+      </c>
       <c r="H45" s="7" t="n">
-        <v>0.1</v>
+        <v>0.005</v>
       </c>
       <c r="I45" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J45" s="8" t="n">
         <f aca="false">IF(H45="","",H45*IF(I45="USD",Parametri!$B$3,IF(I45="GBP",Parametri!$B$4,IF(I45="CNY",Parametri!$B$5,1))))</f>
-        <v>0.086</v>
+        <v>0.0043</v>
       </c>
       <c r="K45" s="4" t="n">
         <f aca="false">C45*Parametri!$B$7</f>
@@ -3403,51 +3475,55 @@
       </c>
       <c r="L45" s="9" t="n">
         <f aca="false">IF(J45="","",J45*K45)</f>
-        <v>0.086</v>
+        <v>0.0043</v>
       </c>
       <c r="M45" s="11" t="s">
         <v>31</v>
       </c>
       <c r="N45" s="4"/>
-      <c r="O45" s="5"/>
+      <c r="O45" s="5" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
-        <v>184</v>
+        <v>152</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C46" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>143</v>
+        <v>20</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>190</v>
-      </c>
-      <c r="G46" s="4"/>
+        <v>191</v>
+      </c>
+      <c r="G46" s="4" t="s">
+        <v>30</v>
+      </c>
       <c r="H46" s="7" t="n">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="I46" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J46" s="8" t="n">
         <f aca="false">IF(H46="","",H46*IF(I46="USD",Parametri!$B$3,IF(I46="GBP",Parametri!$B$4,IF(I46="CNY",Parametri!$B$5,1))))</f>
-        <v>0.086</v>
+        <v>0.215</v>
       </c>
       <c r="K46" s="4" t="n">
         <f aca="false">C46*Parametri!$B$7</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L46" s="9" t="n">
         <f aca="false">IF(J46="","",J46*K46)</f>
-        <v>0.086</v>
+        <v>0.43</v>
       </c>
       <c r="M46" s="11" t="s">
         <v>31</v>
@@ -3457,133 +3533,123 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>184</v>
+        <v>152</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C47" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>143</v>
+        <v>20</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>193</v>
+        <v>82</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>194</v>
+        <v>30</v>
       </c>
       <c r="H47" s="7" t="n">
-        <v>2.39</v>
+        <v>0.005</v>
       </c>
       <c r="I47" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J47" s="8" t="n">
         <f aca="false">IF(H47="","",H47*IF(I47="USD",Parametri!$B$3,IF(I47="GBP",Parametri!$B$4,IF(I47="CNY",Parametri!$B$5,1))))</f>
-        <v>2.0554</v>
+        <v>0.0043</v>
       </c>
       <c r="K47" s="4" t="n">
         <f aca="false">C47*Parametri!$B$7</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L47" s="9" t="n">
         <f aca="false">IF(J47="","",J47*K47)</f>
-        <v>4.1108</v>
-      </c>
-      <c r="M47" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="N47" s="10" t="s">
+        <v>0.0043</v>
+      </c>
+      <c r="M47" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="N47" s="4"/>
+      <c r="O47" s="5"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B48" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="O47" s="5"/>
-    </row>
-    <row r="48" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="B48" s="5" t="s">
+      <c r="C48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="C48" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D48" s="4" t="s">
+      <c r="E48" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="F48" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="E48" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="F48" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="G48" s="4" t="s">
-        <v>138</v>
-      </c>
+      <c r="G48" s="4"/>
       <c r="H48" s="7" t="n">
-        <v>4.54</v>
+        <v>0.1</v>
       </c>
       <c r="I48" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J48" s="8" t="n">
         <f aca="false">IF(H48="","",H48*IF(I48="USD",Parametri!$B$3,IF(I48="GBP",Parametri!$B$4,IF(I48="CNY",Parametri!$B$5,1))))</f>
-        <v>3.9044</v>
+        <v>0.086</v>
       </c>
       <c r="K48" s="4" t="n">
         <f aca="false">C48*Parametri!$B$7</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L48" s="9" t="n">
         <f aca="false">IF(J48="","",J48*K48)</f>
-        <v>15.6176</v>
-      </c>
-      <c r="M48" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="N48" s="10" t="s">
-        <v>200</v>
-      </c>
-      <c r="O48" s="5" t="s">
-        <v>201</v>
-      </c>
+        <v>0.086</v>
+      </c>
+      <c r="M48" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="N48" s="4"/>
+      <c r="O48" s="5"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="C49" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>204</v>
+        <v>150</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="G49" s="4" t="s">
-        <v>194</v>
-      </c>
+        <v>200</v>
+      </c>
+      <c r="G49" s="4"/>
       <c r="H49" s="7" t="n">
-        <v>14.75</v>
+        <v>0.1</v>
       </c>
       <c r="I49" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J49" s="8" t="n">
         <f aca="false">IF(H49="","",H49*IF(I49="USD",Parametri!$B$3,IF(I49="GBP",Parametri!$B$4,IF(I49="CNY",Parametri!$B$5,1))))</f>
-        <v>12.685</v>
+        <v>0.086</v>
       </c>
       <c r="K49" s="4" t="n">
         <f aca="false">C49*Parametri!$B$7</f>
@@ -3591,324 +3657,514 @@
       </c>
       <c r="L49" s="9" t="n">
         <f aca="false">IF(J49="","",J49*K49)</f>
-        <v>12.685</v>
-      </c>
-      <c r="M49" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="N49" s="10" t="s">
-        <v>206</v>
-      </c>
-      <c r="O49" s="5" t="s">
-        <v>207</v>
-      </c>
+        <v>0.086</v>
+      </c>
+      <c r="M49" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="N49" s="4"/>
+      <c r="O49" s="5"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="C50" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="G50" s="4"/>
+        <v>203</v>
+      </c>
+      <c r="G50" s="4" t="s">
+        <v>204</v>
+      </c>
       <c r="H50" s="7" t="n">
-        <v>0.15</v>
+        <v>2.39</v>
       </c>
       <c r="I50" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J50" s="8" t="n">
         <f aca="false">IF(H50="","",H50*IF(I50="USD",Parametri!$B$3,IF(I50="GBP",Parametri!$B$4,IF(I50="CNY",Parametri!$B$5,1))))</f>
-        <v>0.129</v>
+        <v>2.0554</v>
       </c>
       <c r="K50" s="4" t="n">
         <f aca="false">C50*Parametri!$B$7</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L50" s="9" t="n">
         <f aca="false">IF(J50="","",J50*K50)</f>
-        <v>0.129</v>
-      </c>
-      <c r="M50" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="N50" s="4"/>
+        <v>4.1108</v>
+      </c>
+      <c r="M50" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="N50" s="10" t="s">
+        <v>205</v>
+      </c>
       <c r="O50" s="5"/>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="C51" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="F51" s="5" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>194</v>
+        <v>145</v>
       </c>
       <c r="H51" s="7" t="n">
-        <v>0.71</v>
+        <v>4.54</v>
       </c>
       <c r="I51" s="6" t="s">
         <v>23</v>
       </c>
       <c r="J51" s="8" t="n">
         <f aca="false">IF(H51="","",H51*IF(I51="USD",Parametri!$B$3,IF(I51="GBP",Parametri!$B$4,IF(I51="CNY",Parametri!$B$5,1))))</f>
-        <v>0.6106</v>
+        <v>3.9044</v>
       </c>
       <c r="K51" s="4" t="n">
         <f aca="false">C51*Parametri!$B$7</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L51" s="9" t="n">
         <f aca="false">IF(J51="","",J51*K51)</f>
-        <v>0.6106</v>
+        <v>15.6176</v>
       </c>
       <c r="M51" s="4" t="s">
         <v>24</v>
       </c>
       <c r="N51" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="O51" s="5" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B52" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="C52" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="F52" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="O51" s="5"/>
-    </row>
-    <row r="52" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="B52" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="C52" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D52" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="E52" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="F52" s="5" t="s">
-        <v>219</v>
-      </c>
-      <c r="G52" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="H52" s="7"/>
+      <c r="G52" s="4"/>
+      <c r="H52" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="I52" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="J52" s="8" t="str">
+      <c r="J52" s="8" t="n">
         <f aca="false">IF(H52="","",H52*IF(I52="USD",Parametri!$B$3,IF(I52="GBP",Parametri!$B$4,IF(I52="CNY",Parametri!$B$5,1))))</f>
-        <v/>
+        <v>0.86</v>
       </c>
       <c r="K52" s="4" t="n">
         <f aca="false">C52*Parametri!$B$7</f>
         <v>1</v>
       </c>
-      <c r="L52" s="9" t="str">
+      <c r="L52" s="9" t="n">
         <f aca="false">IF(J52="","",J52*K52)</f>
+        <v>0.86</v>
+      </c>
+      <c r="M52" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="N52" s="4"/>
+      <c r="O52" s="5" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B53" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="C53" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="F53" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="G53" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="H53" s="7" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="I53" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J53" s="8" t="n">
+        <f aca="false">IF(H53="","",H53*IF(I53="USD",Parametri!$B$3,IF(I53="GBP",Parametri!$B$4,IF(I53="CNY",Parametri!$B$5,1))))</f>
+        <v>12.685</v>
+      </c>
+      <c r="K53" s="4" t="n">
+        <f aca="false">C53*Parametri!$B$7</f>
+        <v>1</v>
+      </c>
+      <c r="L53" s="9" t="n">
+        <f aca="false">IF(J53="","",J53*K53)</f>
+        <v>12.685</v>
+      </c>
+      <c r="M53" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="N53" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="O53" s="5" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B54" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="C54" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="F54" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="G54" s="4"/>
+      <c r="H54" s="7" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="I54" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J54" s="8" t="n">
+        <f aca="false">IF(H54="","",H54*IF(I54="USD",Parametri!$B$3,IF(I54="GBP",Parametri!$B$4,IF(I54="CNY",Parametri!$B$5,1))))</f>
+        <v>0.129</v>
+      </c>
+      <c r="K54" s="4" t="n">
+        <f aca="false">C54*Parametri!$B$7</f>
+        <v>1</v>
+      </c>
+      <c r="L54" s="9" t="n">
+        <f aca="false">IF(J54="","",J54*K54)</f>
+        <v>0.129</v>
+      </c>
+      <c r="M54" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="N54" s="4"/>
+      <c r="O54" s="5"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B55" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="C55" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="F55" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="G55" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="H55" s="7" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="I55" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J55" s="8" t="n">
+        <f aca="false">IF(H55="","",H55*IF(I55="USD",Parametri!$B$3,IF(I55="GBP",Parametri!$B$4,IF(I55="CNY",Parametri!$B$5,1))))</f>
+        <v>0.6106</v>
+      </c>
+      <c r="K55" s="4" t="n">
+        <f aca="false">C55*Parametri!$B$7</f>
+        <v>1</v>
+      </c>
+      <c r="L55" s="9" t="n">
+        <f aca="false">IF(J55="","",J55*K55)</f>
+        <v>0.6106</v>
+      </c>
+      <c r="M55" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="N55" s="10" t="s">
+        <v>230</v>
+      </c>
+      <c r="O55" s="5"/>
+    </row>
+    <row r="56" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="C56" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="F56" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="H56" s="7"/>
+      <c r="I56" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J56" s="8" t="str">
+        <f aca="false">IF(H56="","",H56*IF(I56="USD",Parametri!$B$3,IF(I56="GBP",Parametri!$B$4,IF(I56="CNY",Parametri!$B$5,1))))</f>
         <v/>
       </c>
-      <c r="M52" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="N52" s="10" t="s">
-        <v>221</v>
-      </c>
-      <c r="O52" s="5" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K54" s="13" t="s">
-        <v>223</v>
-      </c>
-      <c r="L54" s="14" t="n">
-        <f aca="false">SUM(L5:L52)</f>
-        <v>124.4746268</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K55" s="15" t="s">
-        <v>224</v>
-      </c>
-      <c r="L55" s="16" t="n">
-        <f aca="false">SUMIF(M5:M52,"verificato",L5:L52)</f>
-        <v>115.9515268</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K56" s="15" t="s">
-        <v>225</v>
-      </c>
-      <c r="L56" s="16" t="n">
-        <f aca="false">SUMIF(M5:M52,"stima",L5:L52)</f>
-        <v>8.5231</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K57" s="15" t="s">
-        <v>226</v>
-      </c>
-      <c r="L57" s="15" t="n">
-        <f aca="false">COUNTIF(M5:M52,"da quotare")</f>
-        <v>2</v>
+      <c r="K56" s="4" t="n">
+        <f aca="false">C56*Parametri!$B$7</f>
+        <v>1</v>
+      </c>
+      <c r="L56" s="9" t="str">
+        <f aca="false">IF(J56="","",J56*K56)</f>
+        <v/>
+      </c>
+      <c r="M56" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="N56" s="10" t="s">
+        <v>236</v>
+      </c>
+      <c r="O56" s="5" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K58" s="13" t="s">
+        <v>238</v>
+      </c>
+      <c r="L58" s="14" t="n">
+        <f aca="false">SUM(L5:L56)</f>
+        <v>125.7316888</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K59" s="13" t="s">
-        <v>227</v>
+      <c r="K59" s="15" t="s">
+        <v>239</v>
+      </c>
+      <c r="L59" s="16" t="n">
+        <f aca="false">SUMIF(M5:M56,"verificato",L5:L56)</f>
+        <v>116.0088888</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="K60" s="15" t="s">
-        <v>17</v>
+        <v>240</v>
       </c>
       <c r="L60" s="16" t="n">
-        <f aca="false">SUMIF(A5:A52,"Condensatori",L5:L52)</f>
-        <v>0.8365048</v>
+        <f aca="false">SUMIF(M5:M56,"stima",L5:L56)</f>
+        <v>9.7228</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="K61" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="L61" s="16" t="n">
-        <f aca="false">SUMIF(A5:A52,"Diodi",L5:L52)</f>
-        <v>3.349872</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K62" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="L62" s="16" t="n">
-        <f aca="false">SUMIF(A5:A52,"Protezioni",L5:L52)</f>
-        <v>0.39925</v>
+        <v>241</v>
+      </c>
+      <c r="L61" s="15" t="n">
+        <f aca="false">COUNTIF(M5:M56,"da quotare")</f>
+        <v>2</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K63" s="15" t="s">
-        <v>100</v>
-      </c>
-      <c r="L63" s="16" t="n">
-        <f aca="false">SUMIF(A5:A52,"Connettori",L5:L52)</f>
-        <v>3.634</v>
+      <c r="K63" s="13" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="K64" s="15" t="s">
-        <v>120</v>
+        <v>17</v>
       </c>
       <c r="L64" s="16" t="n">
-        <f aca="false">SUMIF(A5:A52,"Modulo WiFi",L5:L52)</f>
-        <v>7.44</v>
+        <f aca="false">SUMIF(A5:A56,"Condensatori",L5:L56)</f>
+        <v>0.9540668</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="K65" s="15" t="s">
-        <v>128</v>
+        <v>62</v>
       </c>
       <c r="L65" s="16" t="n">
-        <f aca="false">SUMIF(A5:A52,"Magnetici",L5:L52)</f>
-        <v>0.258</v>
+        <f aca="false">SUMIF(A5:A56,"Diodi",L5:L56)</f>
+        <v>3.349872</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="K66" s="15" t="s">
-        <v>133</v>
+        <v>83</v>
       </c>
       <c r="L66" s="16" t="n">
-        <f aca="false">SUMIF(A5:A52,"Transistor",L5:L52)</f>
-        <v>61.5416</v>
+        <f aca="false">SUMIF(A5:A56,"Protezioni",L5:L56)</f>
+        <v>0.39925</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="K67" s="15" t="s">
-        <v>145</v>
+        <v>103</v>
       </c>
       <c r="L67" s="16" t="n">
-        <f aca="false">SUMIF(A5:A52,"Resistori",L5:L52)</f>
-        <v>13.6904</v>
+        <f aca="false">SUMIF(A5:A56,"Connettori",L5:L56)</f>
+        <v>3.892</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="K68" s="15" t="s">
-        <v>184</v>
+        <v>127</v>
       </c>
       <c r="L68" s="16" t="n">
-        <f aca="false">SUMIF(A5:A52,"Integrati",L5:L52)</f>
-        <v>33.325</v>
+        <f aca="false">SUMIF(A5:A56,"Modulo WiFi",L5:L56)</f>
+        <v>7.44</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="K69" s="15" t="s">
-        <v>216</v>
+        <v>135</v>
       </c>
       <c r="L69" s="16" t="n">
-        <f aca="false">SUMIF(A5:A52,"PCB",L5:L52)</f>
-        <v>0</v>
+        <f aca="false">SUMIF(A5:A56,"Magnetici",L5:L56)</f>
+        <v>0.258</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K70" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="L70" s="16" t="n">
+        <f aca="false">SUMIF(A5:A56,"Transistor",L5:L56)</f>
+        <v>61.5416</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="K71" s="15" t="s">
-        <v>228</v>
-      </c>
-      <c r="L71" s="17" t="n">
-        <f aca="false">Meccanica!L13</f>
-        <v>22</v>
+        <v>152</v>
+      </c>
+      <c r="L71" s="16" t="n">
+        <f aca="false">SUMIF(A5:A56,"Resistori",L5:L56)</f>
+        <v>13.7119</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K72" s="13" t="s">
-        <v>229</v>
-      </c>
-      <c r="L72" s="14" t="n">
-        <f aca="false">L54+L71</f>
-        <v>146.4746268</v>
+      <c r="K72" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="L72" s="16" t="n">
+        <f aca="false">SUMIF(A5:A56,"Integrati",L5:L56)</f>
+        <v>34.185</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K73" s="15" t="s">
+        <v>231</v>
+      </c>
+      <c r="L73" s="16" t="n">
+        <f aca="false">SUMIF(A5:A56,"PCB",L5:L56)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K75" s="15" t="s">
+        <v>243</v>
+      </c>
+      <c r="L75" s="17" t="n">
+        <f aca="false">Meccanica!L17</f>
+        <v>41.5</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K76" s="13" t="s">
+        <v>244</v>
+      </c>
+      <c r="L76" s="14" t="n">
+        <f aca="false">L58+L75</f>
+        <v>167.2316888</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:O52"/>
+  <autoFilter ref="A4:O56"/>
   <hyperlinks>
     <hyperlink ref="N5" r:id="rId1" display="https://store.comet.bg/en/Catalogue/Product/37095"/>
     <hyperlink ref="N7" r:id="rId2" display="https://www.lcsc.com/product-detail/C93194.html"/>
     <hyperlink ref="N10" r:id="rId3" display="https://www.lcsc.com/product-detail/C93194.html"/>
     <hyperlink ref="N11" r:id="rId4" display="https://www.lcsc.com/category/1142.html"/>
-    <hyperlink ref="N14" r:id="rId5" display="https://www.lcsc.com/product-image/C145332.html"/>
-    <hyperlink ref="N19" r:id="rId6" display="https://uk.rs-online.com/web/p/car-fuses/7874154"/>
-    <hyperlink ref="N27" r:id="rId7" display="https://www.tinytronics.nl/shop/nl/communicatie/wi-fi/wemos-lolin-d1-mini-pro-v2-esp8266-ch340c"/>
-    <hyperlink ref="N29" r:id="rId8" display="https://www.findchips.com/search/H75N1"/>
-    <hyperlink ref="N41" r:id="rId9" display="https://www.element14.cn/en-CN/vishay/wsk2512r0200fea/current-sense-res-0r02-1-1-w-2512/dp/1107431"/>
-    <hyperlink ref="N47" r:id="rId10" display="https://www.flux.ai/lcsc/opa2196idr.md"/>
-    <hyperlink ref="N48" r:id="rId11" display="https://www.digikey.com/en/products/detail/texas-instruments/INA228AIDGST/13691047"/>
-    <hyperlink ref="N49" r:id="rId12" display="https://www.electronicsdatasheets.com/manufacturers/texas-instruments/parts/dac8565"/>
-    <hyperlink ref="N51" r:id="rId13" display="https://www.oemstrade.com/search/ap63205wu-7"/>
-    <hyperlink ref="N52" r:id="rId14" display="https://jlcpcb.com"/>
+    <hyperlink ref="N15" r:id="rId5" display="https://www.lcsc.com/product-image/C145332.html"/>
+    <hyperlink ref="N20" r:id="rId6" display="https://uk.rs-online.com/web/p/car-fuses/7874154"/>
+    <hyperlink ref="N29" r:id="rId7" display="https://www.tinytronics.nl/shop/nl/communicatie/wi-fi/wemos-lolin-d1-mini-pro-v2-esp8266-ch340c"/>
+    <hyperlink ref="N31" r:id="rId8" display="https://www.findchips.com/search/H75N1"/>
+    <hyperlink ref="N43" r:id="rId9" display="https://www.element14.cn/en-CN/vishay/wsk2512r0200fea/current-sense-res-0r02-1-1-w-2512/dp/1107431"/>
+    <hyperlink ref="N50" r:id="rId10" display="https://www.flux.ai/lcsc/opa2196idr.md"/>
+    <hyperlink ref="N51" r:id="rId11" display="https://www.digikey.com/en/products/detail/texas-instruments/INA228AIDGST/13691047"/>
+    <hyperlink ref="N53" r:id="rId12" display="https://www.electronicsdatasheets.com/manufacturers/texas-instruments/parts/dac8565"/>
+    <hyperlink ref="N55" r:id="rId13" display="https://www.oemstrade.com/search/ap63205wu-7"/>
+    <hyperlink ref="N56" r:id="rId14" display="https://jlcpcb.com"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3926,7 +4182,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -3945,7 +4201,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>230</v>
+        <v>245</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3953,13 +4209,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>231</v>
+        <v>246</v>
       </c>
       <c r="C3" s="18" t="s">
         <v>4</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>232</v>
+        <v>247</v>
       </c>
       <c r="E3" s="18" t="s">
         <v>9</v>
@@ -3988,10 +4244,10 @@
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>233</v>
+        <v>248</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>234</v>
+        <v>249</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>1</v>
@@ -3999,14 +4255,14 @@
       <c r="D4" s="4"/>
       <c r="E4" s="6"/>
       <c r="F4" s="6" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="5" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="J4" s="19" t="str">
         <f aca="false">IF(E4="","",E4*IF(F4="USD",Parametri!$B$3,IF(F4="GBP",Parametri!$B$4,IF(F4="CNY",Parametri!$B$5,1))))</f>
@@ -4023,10 +4279,10 @@
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>233</v>
+        <v>248</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>236</v>
+        <v>251</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>1</v>
@@ -4034,14 +4290,14 @@
       <c r="D5" s="4"/>
       <c r="E5" s="6"/>
       <c r="F5" s="6" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="H5" s="4"/>
       <c r="I5" s="5" t="s">
-        <v>237</v>
+        <v>252</v>
       </c>
       <c r="J5" s="19" t="str">
         <f aca="false">IF(E5="","",E5*IF(F5="USD",Parametri!$B$3,IF(F5="GBP",Parametri!$B$4,IF(F5="CNY",Parametri!$B$5,1))))</f>
@@ -4058,10 +4314,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>233</v>
+        <v>248</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>238</v>
+        <v>253</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>1</v>
@@ -4069,14 +4325,14 @@
       <c r="D6" s="4"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="H6" s="4"/>
       <c r="I6" s="5" t="s">
-        <v>239</v>
+        <v>254</v>
       </c>
       <c r="J6" s="19" t="str">
         <f aca="false">IF(E6="","",E6*IF(F6="USD",Parametri!$B$3,IF(F6="GBP",Parametri!$B$4,IF(F6="CNY",Parametri!$B$5,1))))</f>
@@ -4093,10 +4349,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>233</v>
+        <v>248</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>240</v>
+        <v>255</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>2</v>
@@ -4106,7 +4362,7 @@
         <v>0.5</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="G7" s="11" t="s">
         <v>31</v>
@@ -4128,10 +4384,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>233</v>
+        <v>248</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>241</v>
+        <v>256</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>1</v>
@@ -4141,7 +4397,7 @@
         <v>5</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="G8" s="11" t="s">
         <v>31</v>
@@ -4163,22 +4419,22 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>242</v>
+        <v>257</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>243</v>
+        <v>258</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>244</v>
+        <v>259</v>
       </c>
       <c r="E9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="G9" s="11" t="s">
         <v>31</v>
@@ -4200,10 +4456,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>245</v>
+        <v>260</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>246</v>
+        <v>261</v>
       </c>
       <c r="C10" s="6" t="n">
         <v>1</v>
@@ -4213,7 +4469,7 @@
         <v>10</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="G10" s="11" t="s">
         <v>31</v>
@@ -4233,31 +4489,33 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>120</v>
+        <v>262</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
       <c r="C11" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="6" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="G11" s="11" t="s">
         <v>31</v>
       </c>
       <c r="H11" s="4"/>
-      <c r="I11" s="5"/>
+      <c r="I11" s="5" t="s">
+        <v>264</v>
+      </c>
       <c r="J11" s="19" t="n">
         <f aca="false">IF(E11="","",E11*IF(F11="USD",Parametri!$B$3,IF(F11="GBP",Parametri!$B$4,IF(F11="CNY",Parametri!$B$5,1))))</f>
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="K11" s="20" t="n">
         <f aca="false">C11*Parametri!$B$7</f>
@@ -4265,16 +4523,158 @@
       </c>
       <c r="L11" s="19" t="n">
         <f aca="false">IF(J11="","",J11*K11)</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="4"/>
+      <c r="E12" s="6" t="n">
         <v>3</v>
       </c>
+      <c r="F12" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="H12" s="4"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="19" t="n">
+        <f aca="false">IF(E12="","",E12*IF(F12="USD",Parametri!$B$3,IF(F12="GBP",Parametri!$B$4,IF(F12="CNY",Parametri!$B$5,1))))</f>
+        <v>3</v>
+      </c>
+      <c r="K12" s="20" t="n">
+        <f aca="false">C12*Parametri!$B$7</f>
+        <v>1</v>
+      </c>
+      <c r="L12" s="19" t="n">
+        <f aca="false">IF(J12="","",J12*K12)</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="K13" s="13" t="s">
-        <v>228</v>
-      </c>
-      <c r="L13" s="14" t="n">
-        <f aca="false">SUM(L4:L11)</f>
-        <v>22</v>
+      <c r="A13" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="4"/>
+      <c r="E13" s="6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="H13" s="4"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="19" t="n">
+        <f aca="false">IF(E13="","",E13*IF(F13="USD",Parametri!$B$3,IF(F13="GBP",Parametri!$B$4,IF(F13="CNY",Parametri!$B$5,1))))</f>
+        <v>2.5</v>
+      </c>
+      <c r="K13" s="20" t="n">
+        <f aca="false">C13*Parametri!$B$7</f>
+        <v>1</v>
+      </c>
+      <c r="L13" s="19" t="n">
+        <f aca="false">IF(J13="","",J13*K13)</f>
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="4"/>
+      <c r="E14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="H14" s="4"/>
+      <c r="I14" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="J14" s="19" t="n">
+        <f aca="false">IF(E14="","",E14*IF(F14="USD",Parametri!$B$3,IF(F14="GBP",Parametri!$B$4,IF(F14="CNY",Parametri!$B$5,1))))</f>
+        <v>2</v>
+      </c>
+      <c r="K14" s="20" t="n">
+        <f aca="false">C14*Parametri!$B$7</f>
+        <v>1</v>
+      </c>
+      <c r="L14" s="19" t="n">
+        <f aca="false">IF(J14="","",J14*K14)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="4"/>
+      <c r="E15" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="H15" s="4"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="19" t="n">
+        <f aca="false">IF(E15="","",E15*IF(F15="USD",Parametri!$B$3,IF(F15="GBP",Parametri!$B$4,IF(F15="CNY",Parametri!$B$5,1))))</f>
+        <v>3</v>
+      </c>
+      <c r="K15" s="20" t="n">
+        <f aca="false">C15*Parametri!$B$7</f>
+        <v>1</v>
+      </c>
+      <c r="L15" s="19" t="n">
+        <f aca="false">IF(J15="","",J15*K15)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K17" s="13" t="s">
+        <v>243</v>
+      </c>
+      <c r="L17" s="14" t="n">
+        <f aca="false">SUM(L4:L15)</f>
+        <v>41.5</v>
       </c>
     </row>
   </sheetData>
@@ -4303,40 +4703,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>248</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="15" t="s">
-        <v>249</v>
+        <v>271</v>
       </c>
       <c r="B3" s="21" t="n">
         <v>0.86</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>250</v>
+        <v>272</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>251</v>
+        <v>273</v>
       </c>
       <c r="B4" s="21" t="n">
         <v>1.15</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>252</v>
+        <v>274</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>253</v>
+        <v>275</v>
       </c>
       <c r="B5" s="21" t="n">
         <v>0.12</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>254</v>
+        <v>276</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4345,13 +4745,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>255</v>
+        <v>277</v>
       </c>
       <c r="B7" s="22" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>256</v>
+        <v>278</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4363,77 +4763,77 @@
     </row>
     <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="24" t="s">
-        <v>257</v>
+        <v>279</v>
       </c>
       <c r="B11" s="24"/>
       <c r="C11" s="24"/>
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="24" t="s">
-        <v>258</v>
+        <v>280</v>
       </c>
       <c r="B12" s="24"/>
       <c r="C12" s="24"/>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="24" t="s">
-        <v>259</v>
+        <v>281</v>
       </c>
       <c r="B13" s="24"/>
       <c r="C13" s="24"/>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="24" t="s">
-        <v>260</v>
+        <v>282</v>
       </c>
       <c r="B14" s="24"/>
       <c r="C14" s="24"/>
     </row>
     <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="24" t="s">
-        <v>261</v>
+        <v>283</v>
       </c>
       <c r="B15" s="24"/>
       <c r="C15" s="24"/>
     </row>
     <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="24" t="s">
-        <v>262</v>
+        <v>284</v>
       </c>
       <c r="B16" s="24"/>
       <c r="C16" s="24"/>
     </row>
     <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="24" t="s">
-        <v>263</v>
+        <v>285</v>
       </c>
       <c r="B17" s="24"/>
       <c r="C17" s="24"/>
     </row>
     <row r="18" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="24" t="s">
-        <v>264</v>
+        <v>286</v>
       </c>
       <c r="B18" s="24"/>
       <c r="C18" s="24"/>
     </row>
     <row r="19" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="24" t="s">
-        <v>265</v>
+        <v>287</v>
       </c>
       <c r="B19" s="24"/>
       <c r="C19" s="24"/>
     </row>
     <row r="20" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="24" t="s">
-        <v>266</v>
+        <v>288</v>
       </c>
       <c r="B20" s="24"/>
       <c r="C20" s="24"/>
     </row>
     <row r="21" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="24" t="s">
-        <v>267</v>
+        <v>289</v>
       </c>
       <c r="B21" s="24"/>
       <c r="C21" s="24"/>

</xml_diff>